<commit_message>
prg Fri Jun  5 12:37:18 PM CEST 2026
</commit_message>
<xml_diff>
--- a/public/routers/A0_Sistema_FV/A61_Conectado_a_red/FV05_pvgis.xlsx
+++ b/public/routers/A0_Sistema_FV/A61_Conectado_a_red/FV05_pvgis.xlsx
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>..</t>
+          <t>~</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -2127,17 +2127,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>..Otrsos</t>
+          <t>~Otrsos</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>..Otdros</t>
+          <t>~Otdros</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>..Otros</t>
+          <t>~Otros</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -2154,7 +2154,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>..€</t>
+          <t>~€</t>
         </is>
       </c>
     </row>
@@ -2528,12 +2528,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>..Otros</t>
+          <t>~Otros</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>..Otros</t>
+          <t>~Otros</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -2550,7 +2550,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>..€</t>
+          <t>~€</t>
         </is>
       </c>
     </row>

</xml_diff>